<commit_message>
Tighten viewer supplier privacy and export selection
</commit_message>
<xml_diff>
--- a/public/导入模板.xlsx
+++ b/public/导入模板.xlsx
@@ -268,7 +268,7 @@
     <t>是</t>
   </si>
   <si>
-    <t>产品组的唯一编号，同一产品多个规格时请重复填写此SKU</t>
+    <t>产品组的唯一编号。不同产品必须使用不同产品组SKU；同一产品多个规格时，可每行重复填写此SKU，也可只在第一行填写、后续连续规格行留空</t>
   </si>
   <si>
     <t>否</t>
@@ -277,10 +277,10 @@
     <t>产品图片。支持：1) 网络URL（多张用逗号/分号分隔）；2) 直接复制粘贴图片到单元格；3) 两者混合使用。同一产品多规格时只在第一行填写</t>
   </si>
   <si>
-    <t>产品显示名称（同一产品多规格时只在第一行填写）</t>
-  </si>
-  <si>
-    <t>供应商名称，如不存在会自动创建</t>
+    <t>产品显示名称。同一产品多个规格时，可每行重复填写，也可只在第一行填写、后续连续规格行留空；同一产品组SKU不能对应多个不同产品名称</t>
+  </si>
+  <si>
+    <t>供应商名称，如不存在会自动创建。同一产品多个规格时，可每行重复填写，也可只在第一行填写、后续连续规格行留空</t>
   </si>
   <si>
     <t>规格描述文字</t>
@@ -295,7 +295,7 @@
     <t>原厂配件编号</t>
   </si>
   <si>
-    <t>进货成本价格（填数字即可）</t>
+    <t>进货成本价格（填数字即可）。导入旧表时，列名为“产品价格”或“产品价格(元)”也会识别为拿货价格</t>
   </si>
   <si>
     <t>对外销售价格（填数字即可）</t>
@@ -304,7 +304,7 @@
     <t>适用的车型名称</t>
   </si>
   <si>
-    <t>产品来源链接（网址）</t>
+    <t>产品来源链接，建议填写 http:// 或 https:// 开头的网址。同一产品多个规格时只在第一行填写；后续连续规格行留空会继承第一行链接</t>
   </si>
   <si>
     <t>单个产品净重</t>
@@ -355,7 +355,7 @@
     <t>混合使用</t>
   </si>
   <si>
-    <t>URL和嵌入图片可同时使用，系统会合并所有图片来源。最多20张</t>
+    <t>URL和嵌入图片可同时使用，系统会合并所有图片来源</t>
   </si>
   <si>
     <t>注意</t>
@@ -909,7 +909,7 @@
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Add AI instructions to import template
</commit_message>
<xml_diff>
--- a/public/导入模板.xlsx
+++ b/public/导入模板.xlsx
@@ -6,6 +6,7 @@
   <sheets>
     <sheet sheetId="1" name="导入模板" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="填写说明" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="AI填写说明" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -104,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="126">
   <si>
     <t>产品组SKU</t>
   </si>
@@ -365,6 +366,123 @@
   </si>
   <si>
     <t>同一产品有多个规格时，只在第一行填写图片URL或粘贴图片，后续规格行留空即可</t>
+  </si>
+  <si>
+    <t>步骤/场景</t>
+  </si>
+  <si>
+    <t>AI需要遵守的要求</t>
+  </si>
+  <si>
+    <t>常见错误/处理方式</t>
+  </si>
+  <si>
+    <t>总体目标</t>
+  </si>
+  <si>
+    <t>把任意来源表整理成“导入模板”工作表的列结构。每一行代表一个产品规格；同一产品有多个规格时，使用同一个产品组SKU。只填写能从源数据确认的信息。</t>
+  </si>
+  <si>
+    <t>不要为了凑完整而编造价格、链接、尺寸、重量、适配车型、OE码或图片。源表没有就留空。</t>
+  </si>
+  <si>
+    <t>识别源表表头</t>
+  </si>
+  <si>
+    <t>源数据表头不一定在第1行，先在前20行寻找类似产品名称、SKU/编号、供应商、规格、价格、车型、链接等字段。合并单元格或空白延续行要按上下文向下填充，但只能在同一产品范围内填充。</t>
+  </si>
+  <si>
+    <t>不要把标题、说明行、合计行、空白分隔行当成产品数据导入。</t>
+  </si>
+  <si>
+    <t>不同产品必须使用不同产品组SKU；同一产品多个规格必须使用同一个产品组SKU。若源表已有产品组编号则沿用；若只有规格SKU，可为产品组生成稳定编号，例如供应商前缀+连续编号。推荐每个规格行都重复填写产品组SKU，减少歧义。</t>
+  </si>
+  <si>
+    <t>绝不能让同一个产品组SKU对应多个不同产品名称，否则系统会把不同产品合并到一起。</t>
+  </si>
+  <si>
+    <t>填写清晰的产品显示名称。同一产品多个规格的产品名称必须完全一致。推荐每个规格行重复填写产品名称；也可以只在同一产品的第一行填写、后续连续规格行留空。</t>
+  </si>
+  <si>
+    <t>不要把规格、车型、颜色等全部塞进产品名称；这些信息优先放入产品规格或适配车型。</t>
+  </si>
+  <si>
+    <t>供应商为必填。源表有供应商名称时照填；同一产品多规格可每行重复填写。若源表按文件或工作表区分供应商，应把该供应商填入每一行。</t>
+  </si>
+  <si>
+    <t>不要把平台名、店铺链接、联系人误填为供应商，除非源数据明确它就是供应商名称。</t>
+  </si>
+  <si>
+    <t>规格与规格SKU</t>
+  </si>
+  <si>
+    <t>每个规格占一行。规格SKU每行必须填写，优先使用源表规格SKU/商品编号/工厂编号；如果缺失，可基于产品组SKU生成唯一规格SKU，例如 ZFLM-00001-01、ZFLM-00001-02。产品规格填写颜色、左右、型号、针脚、版本等规格差异。</t>
+  </si>
+  <si>
+    <t>同一产品组下规格SKU不能重复。不要把多个规格写在同一个单元格里。</t>
+  </si>
+  <si>
+    <t>价格字段</t>
+  </si>
+  <si>
+    <t>源表中的拿货价、成本价、采购价、产品价格通常填入“拿货价格(元)”；销售价、零售价、对外价填入“销售价格(元)”。尽量只填数字或简单文本，保留小数。</t>
+  </si>
+  <si>
+    <t>不要把区间价、批发阶梯价随意取平均；无法确定单价时可留空或保留源文本说明。</t>
+  </si>
+  <si>
+    <t>OE码和适配车型</t>
+  </si>
+  <si>
+    <t>OE码填原厂编号，可多个编号用逗号、分号或换行分隔。适配车型填品牌、车型、年份、底盘代号等可读信息。</t>
+  </si>
+  <si>
+    <t>不要把OE码写进适配车型，也不要删除前导0或特殊字符。</t>
+  </si>
+  <si>
+    <t>产品链接填写来源商品页，建议为 http:// 或 https:// 开头的网址。同一产品多规格通常只在第一行填写；也可以每个规格行重复填写相同链接。</t>
+  </si>
+  <si>
+    <t>不要把普通英文标题、搜索词或图片链接填入产品链接。没有明确来源链接就留空。</t>
+  </si>
+  <si>
+    <t>图片URL只填写可直接访问的图片地址，支持多张图片用逗号、分号或换行分隔。若源表有嵌入图片，可保留图片在对应产品第一行附近；同一产品多规格只在第一行放图片或图片URL。</t>
+  </si>
+  <si>
+    <t>不要把商品详情页链接填入图片URL。WPS的 =DISPIMG() 公式不等于真实图片URL，不能当URL填写。</t>
+  </si>
+  <si>
+    <t>重量、尺寸、装箱数</t>
+  </si>
+  <si>
+    <t>产品重量/尺寸表示单品信息；包装重量/尺寸表示含包装信息；装箱数表示每箱数量。单位可保留在文本中，例如 13kg、70*40*60。</t>
+  </si>
+  <si>
+    <t>不要把包装重量写到产品重量里；无法判断单品还是包装时保留源表原文并尽量放到更接近的列。</t>
+  </si>
+  <si>
+    <t>备注只放无法归类但对人工复核有用的信息，例如源表注释、特殊条件、需确认事项。</t>
+  </si>
+  <si>
+    <t>不要把必填字段缺失原因藏在备注里；产品组SKU、产品名称、供应商、规格SKU仍应按规则填写。</t>
+  </si>
+  <si>
+    <t>数据类型</t>
+  </si>
+  <si>
+    <t>SKU、OE码、链接、尺寸等按文本处理；价格可填数字。复制公式单元格时使用显示结果，不要写入Excel公式。保留前导0、横线、斜杠、括号等编号字符。</t>
+  </si>
+  <si>
+    <t>不要让Excel自动把长编号转科学计数法，或把 00123 变成 123。</t>
+  </si>
+  <si>
+    <t>导入前自检</t>
+  </si>
+  <si>
+    <t>检查四件事：1) 每行有规格SKU；2) 每个产品组SKU只对应一个产品名称；3) 不同产品没有复用同一产品组SKU；4) 图片URL与产品链接没有混填。</t>
+  </si>
+  <si>
+    <t>发现源数据疑似串行、合并单元格错位或产品边界不清时，宁可留空或标注待确认，不要强行合并。</t>
   </si>
 </sst>
 </file>
@@ -425,7 +543,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -441,6 +559,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1287,4 +1411,185 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="78" customWidth="1"/>
+    <col min="3" max="3" width="58" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="13" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="14" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add product stock and listing controls
</commit_message>
<xml_diff>
--- a/public/导入模板.xlsx
+++ b/public/导入模板.xlsx
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="137">
   <si>
     <t>产品组SKU</t>
   </si>
@@ -119,6 +119,12 @@
     <t>供应商</t>
   </si>
   <si>
+    <t>期货/现货</t>
+  </si>
+  <si>
+    <t>上架时间</t>
+  </si>
+  <si>
     <t>产品规格</t>
   </si>
   <si>
@@ -170,6 +176,12 @@
     <t>博世汽车配件</t>
   </si>
   <si>
+    <t>现货</t>
+  </si>
+  <si>
+    <t>2026-07-29 09:00</t>
+  </si>
+  <si>
     <t>前轮陶瓷片 标准型</t>
   </si>
   <si>
@@ -227,6 +239,12 @@
     <t>广州汽配城A区</t>
   </si>
   <si>
+    <t>期货</t>
+  </si>
+  <si>
+    <t>2026-07-28 14:30</t>
+  </si>
+  <si>
     <t>标准过滤精度 30μm</t>
   </si>
   <si>
@@ -284,6 +302,12 @@
     <t>供应商名称，如不存在会自动创建。同一产品多个规格时，可每行重复填写，也可只在第一行填写、后续连续规格行留空</t>
   </si>
   <si>
+    <t>填写“现货”或“期货”。留空时新产品默认按“现货”处理；同一产品多个规格时只需在第一行填写</t>
+  </si>
+  <si>
+    <t>产品上架日期和时间，推荐格式为 YYYY-MM-DD HH:mm；留空时使用导入时间</t>
+  </si>
+  <si>
     <t>规格描述文字</t>
   </si>
   <si>
@@ -411,6 +435,15 @@
   </si>
   <si>
     <t>不要把平台名、店铺链接、联系人误填为供应商，除非源数据明确它就是供应商名称。</t>
+  </si>
+  <si>
+    <t>期货/现货与上架时间</t>
+  </si>
+  <si>
+    <t>期货/现货只填写“现货”或“期货”。上架时间推荐使用 YYYY-MM-DD HH:mm；源数据没有明确上架时间时留空，让系统使用导入时间。</t>
+  </si>
+  <si>
+    <t>不要根据库存数量猜测期货或现货，也不要把交货周期、采购日期误填成上架时间。</t>
   </si>
   <si>
     <t>规格与规格SKU</t>
@@ -904,28 +937,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="26" customWidth="1"/>
-    <col min="11" max="11" width="30" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="26" customWidth="1"/>
+    <col min="13" max="13" width="30" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
     <col min="15" max="15" width="16" customWidth="1"/>
     <col min="16" max="16" width="12" customWidth="1"/>
-    <col min="17" max="17" width="28" customWidth="1"/>
+    <col min="17" max="17" width="16" customWidth="1"/>
+    <col min="18" max="18" width="12" customWidth="1"/>
+    <col min="19" max="19" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -977,164 +1011,188 @@
       <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" ht="22" customHeight="1" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" s="3">
+        <v>85</v>
+      </c>
+      <c r="K2" s="3">
+        <v>168</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:19" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" s="4">
+        <v>120</v>
+      </c>
+      <c r="K3" s="4">
+        <v>238</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:19" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J4" s="3">
         <v>22</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H2" s="3">
-        <v>85</v>
-      </c>
-      <c r="I2" s="3">
-        <v>168</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="H3" s="4">
-        <v>120</v>
-      </c>
-      <c r="I3" s="4">
-        <v>238</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="O3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q3" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="K4" s="3">
+        <v>45</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="M4" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="H4" s="3">
-        <v>22</v>
-      </c>
-      <c r="I4" s="3">
-        <v>45</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>45</v>
-      </c>
       <c r="N4" s="3" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>49</v>
+        <v>53</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1146,7 +1204,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1156,13 +1214,13 @@
   <sheetData>
     <row r="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1170,10 +1228,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1181,10 +1239,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1192,10 +1250,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1203,10 +1261,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1214,10 +1272,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1225,10 +1283,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1236,10 +1294,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1247,10 +1305,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1258,10 +1316,10 @@
         <v>8</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1269,10 +1327,10 @@
         <v>9</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1280,10 +1338,10 @@
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1291,10 +1349,10 @@
         <v>11</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1302,10 +1360,10 @@
         <v>12</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1313,10 +1371,10 @@
         <v>13</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1324,10 +1382,10 @@
         <v>14</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1335,10 +1393,10 @@
         <v>15</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -1346,65 +1404,87 @@
         <v>16</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>73</v>
+        <v>17</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>86</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1415,7 +1495,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1425,35 +1505,35 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1461,10 +1541,10 @@
         <v>0</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
@@ -1472,10 +1552,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1483,109 +1563,120 @@
         <v>3</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>10</v>
+        <v>119</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>115</v>
+        <v>1</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
     </row>
     <row r="13" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>16</v>
+        <v>126</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>120</v>
+        <v>18</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" ht="56" customHeight="1" spans="1:3" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>125</v>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" ht="56" customHeight="1" spans="1:3" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>